<commit_message>
update scripts for figures of case
</commit_message>
<xml_diff>
--- a/result/case/case1.xlsx
+++ b/result/case/case1.xlsx
@@ -634,7 +634,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -667,14 +667,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>hoval</t>
+          <t>inc</t>
         </is>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0.4998785577643763</v>
       </c>
       <c r="D2">
-        <v>-0</v>
+        <v>0.0002551500451938893</v>
       </c>
     </row>
     <row r="3">
@@ -685,32 +685,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>inc</t>
+          <t>crime</t>
         </is>
       </c>
       <c r="C3">
-        <v>0.4998785577643763</v>
+        <v>-0.5744867471853496</v>
       </c>
       <c r="D3">
-        <v>0.0002551500451938893</v>
+        <v>3.17010026723608E-05</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>hoval</t>
+          <t>inc</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>crime</t>
+          <t>hoval</t>
         </is>
       </c>
       <c r="C4">
-        <v>-0.5744867471853496</v>
+        <v>0.4998785577643763</v>
       </c>
       <c r="D4">
-        <v>3.17010026723608E-05</v>
+        <v>0.0002551500451938893</v>
       </c>
     </row>
     <row r="5">
@@ -721,104 +721,50 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>hoval</t>
+          <t>crime</t>
         </is>
       </c>
       <c r="C5">
-        <v>0.4998785577643763</v>
+        <v>-0.6955897734584623</v>
       </c>
       <c r="D5">
-        <v>0.0002551500451938893</v>
+        <v>8.703075025936445E-08</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>inc</t>
+          <t>crime</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>inc</t>
+          <t>hoval</t>
         </is>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>-0.5744867471853496</v>
       </c>
       <c r="D6">
-        <v>-0</v>
+        <v>1.58505013361804E-05</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>inc</t>
+          <t>crime</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>crime</t>
+          <t>inc</t>
         </is>
       </c>
       <c r="C7">
         <v>-0.6955897734584623</v>
       </c>
       <c r="D7">
-        <v>8.703075025936445E-08</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>crime</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>hoval</t>
-        </is>
-      </c>
-      <c r="C8">
-        <v>-0.5744867471853496</v>
-      </c>
-      <c r="D8">
-        <v>1.58505013361804E-05</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>crime</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>inc</t>
-        </is>
-      </c>
-      <c r="C9">
-        <v>-0.6955897734584623</v>
-      </c>
-      <c r="D9">
         <v>2.901025008645482E-08</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>crime</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>crime</t>
-        </is>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10">
-        <v>-0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update results and figures for case studies
</commit_message>
<xml_diff>
--- a/result/case/case1.xlsx
+++ b/result/case/case1.xlsx
@@ -391,10 +391,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.1929012345679012</v>
+        <v>0.07439999999999999</v>
       </c>
       <c r="D2">
-        <v>5.474672474409928E-05</v>
+        <v>7.804437058098957E-28</v>
       </c>
     </row>
     <row r="3">
@@ -409,10 +409,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.2469135802469136</v>
+        <v>0.1336</v>
       </c>
       <c r="D3">
-        <v>0.004864208186179272</v>
+        <v>8.589914961212566E-12</v>
       </c>
     </row>
     <row r="4">
@@ -427,10 +427,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.1095679012345679</v>
+        <v>0.0472</v>
       </c>
       <c r="D4">
-        <v>3.08794865172942E-10</v>
+        <v>1.512896130081941E-42</v>
       </c>
     </row>
     <row r="5">
@@ -445,10 +445,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.1234567901234568</v>
+        <v>0.0464</v>
       </c>
       <c r="D5">
-        <v>4.804442753242007E-09</v>
+        <v>1.582279896822512E-44</v>
       </c>
     </row>
     <row r="6">
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.1728395061728395</v>
+        <v>0.0696</v>
       </c>
       <c r="D6">
-        <v>7.587769234624996E-06</v>
+        <v>1.250759598003088E-29</v>
       </c>
     </row>
     <row r="7">
@@ -481,10 +481,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.2561728395061729</v>
+        <v>0.1152</v>
       </c>
       <c r="D7">
-        <v>0.007722215987824777</v>
+        <v>9.128475680692894E-15</v>
       </c>
     </row>
   </sheetData>
@@ -531,10 +531,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.2372003598376317</v>
+        <v>0.2409946417943775</v>
       </c>
       <c r="D2">
-        <v>0.1007863699619085</v>
+        <v>0.09529596052654821</v>
       </c>
     </row>
     <row r="3">
@@ -549,10 +549,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.6419288059776628</v>
+        <v>0.5758561426755622</v>
       </c>
       <c r="D3">
-        <v>6.657865290193854E-07</v>
+        <v>1.496551076263231E-05</v>
       </c>
     </row>
     <row r="4">
@@ -567,10 +567,10 @@
         </is>
       </c>
       <c r="C4">
-        <v>0.4077414146794142</v>
+        <v>0.4016465624792653</v>
       </c>
       <c r="D4">
-        <v>0.003636923169701767</v>
+        <v>0.004230060809255809</v>
       </c>
     </row>
     <row r="5">
@@ -585,10 +585,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.6018242990998784</v>
+        <v>0.5611671771902005</v>
       </c>
       <c r="D5">
-        <v>4.78484692201242E-06</v>
+        <v>2.735352199456642E-05</v>
       </c>
     </row>
     <row r="6">
@@ -603,10 +603,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.1981525002572533</v>
+        <v>0.2264557778720811</v>
       </c>
       <c r="D6">
-        <v>0.1723041877953277</v>
+        <v>0.1176598148571866</v>
       </c>
     </row>
     <row r="7">
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.3556509555148407</v>
+        <v>0.3630723600274959</v>
       </c>
       <c r="D7">
-        <v>0.01214582219349691</v>
+        <v>0.01034582954412855</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update case figures and results
</commit_message>
<xml_diff>
--- a/result/case/case1.xlsx
+++ b/result/case/case1.xlsx
@@ -391,10 +391,10 @@
         </is>
       </c>
       <c r="C2">
-        <v>0.07439999999999999</v>
+        <v>0.0808</v>
       </c>
       <c r="D2">
-        <v>7.804437058098957E-28</v>
+        <v>8.072164768242996E-23</v>
       </c>
     </row>
     <row r="3">
@@ -409,10 +409,10 @@
         </is>
       </c>
       <c r="C3">
-        <v>0.1336</v>
+        <v>0.1432</v>
       </c>
       <c r="D3">
-        <v>8.589914961212566E-12</v>
+        <v>1.022037555902064E-10</v>
       </c>
     </row>
     <row r="4">
@@ -445,10 +445,10 @@
         </is>
       </c>
       <c r="C5">
-        <v>0.0464</v>
+        <v>0.0496</v>
       </c>
       <c r="D5">
-        <v>1.582279896822512E-44</v>
+        <v>7.690666776785052E-43</v>
       </c>
     </row>
     <row r="6">
@@ -463,10 +463,10 @@
         </is>
       </c>
       <c r="C6">
-        <v>0.0696</v>
+        <v>0.076</v>
       </c>
       <c r="D6">
-        <v>1.250759598003088E-29</v>
+        <v>6.514867964944103E-24</v>
       </c>
     </row>
     <row r="7">
@@ -481,10 +481,10 @@
         </is>
       </c>
       <c r="C7">
-        <v>0.1152</v>
+        <v>0.1176</v>
       </c>
       <c r="D7">
-        <v>9.128475680692894E-15</v>
+        <v>4.461943622118817E-14</v>
       </c>
     </row>
   </sheetData>
@@ -534,7 +534,7 @@
         <v>0.2409946417943775</v>
       </c>
       <c r="D2">
-        <v>0.09529596052654821</v>
+        <v>0.09529596052654807</v>
       </c>
     </row>
     <row r="3">
@@ -552,7 +552,7 @@
         <v>0.5758561426755622</v>
       </c>
       <c r="D3">
-        <v>1.496551076263231E-05</v>
+        <v>1.496551076251382E-05</v>
       </c>
     </row>
     <row r="4">
@@ -570,7 +570,7 @@
         <v>0.4016465624792653</v>
       </c>
       <c r="D4">
-        <v>0.004230060809255809</v>
+        <v>0.004230060809255795</v>
       </c>
     </row>
     <row r="5">
@@ -588,7 +588,7 @@
         <v>0.5611671771902005</v>
       </c>
       <c r="D5">
-        <v>2.735352199456642E-05</v>
+        <v>2.735352199453464E-05</v>
       </c>
     </row>
     <row r="6">
@@ -624,7 +624,7 @@
         <v>0.3630723600274959</v>
       </c>
       <c r="D7">
-        <v>0.01034582954412855</v>
+        <v>0.0103458295441285</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update case results and figures
</commit_message>
<xml_diff>
--- a/result/case/case1.xlsx
+++ b/result/case/case1.xlsx
@@ -370,7 +370,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ca</t>
+          <t>cs</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ca</t>
+          <t>cs</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -650,7 +650,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ca</t>
+          <t>cs</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ca</t>
+          <t>cs</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
sync update with spEDM 1.8
</commit_message>
<xml_diff>
--- a/result/case/case1.xlsx
+++ b/result/case/case1.xlsx
@@ -534,7 +534,7 @@
         <v>0.2409946417943777</v>
       </c>
       <c r="D2">
-        <v>0.09529596052654772</v>
+        <v>0.09529596052654776</v>
       </c>
     </row>
     <row r="3">
@@ -552,7 +552,7 @@
         <v>0.5758561426755622</v>
       </c>
       <c r="D3">
-        <v>1.496551076251382E-05</v>
+        <v>1.496551076263231E-05</v>
       </c>
     </row>
     <row r="4">
@@ -588,7 +588,7 @@
         <v>0.5611671771902004</v>
       </c>
       <c r="D5">
-        <v>2.735352199453475E-05</v>
+        <v>2.735352199456642E-05</v>
       </c>
     </row>
     <row r="6">
@@ -606,7 +606,7 @@
         <v>0.2264557778720812</v>
       </c>
       <c r="D6">
-        <v>0.1176598148571865</v>
+        <v>0.1176598148571866</v>
       </c>
     </row>
     <row r="7">
@@ -624,7 +624,7 @@
         <v>0.3630723600274957</v>
       </c>
       <c r="D7">
-        <v>0.01034582954412856</v>
+        <v>0.01034582954412855</v>
       </c>
     </row>
   </sheetData>

</xml_diff>